<commit_message>
fix: set processor to Novastar for all displays (remove TBD)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/COAT-Specs-FILLED.xlsx
+++ b/docs/COAT-Specs-FILLED.xlsx
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3748" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3748" uniqueCount="189">
   <si>
     <t>Capital One Arena — Product Data Forms (Filled)</t>
   </si>
@@ -352,7 +352,7 @@
     <t>OEM PROCESSOR MANUFACTURER:</t>
   </si>
   <si>
-    <t>TBD — Pending confirmation from Eric</t>
+    <t>Novastar</t>
   </si>
   <si>
     <t>FACTORY PRODUCING LED MODULES:</t>
@@ -514,9 +514,6 @@
   </si>
   <si>
     <t>LG GSQA083</t>
-  </si>
-  <si>
-    <t>Novastar</t>
   </si>
   <si>
     <t>LG Yaham, China</t>
@@ -2111,7 +2108,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -2120,7 +2117,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -2185,7 +2182,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -2690,7 +2687,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -2810,7 +2807,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -2819,7 +2816,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -2884,7 +2881,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -3389,7 +3386,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -3509,7 +3506,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -3518,7 +3515,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -3583,7 +3580,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -4088,7 +4085,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -4208,7 +4205,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -4217,7 +4214,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -4282,7 +4279,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -4787,7 +4784,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -4907,7 +4904,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -4916,7 +4913,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -4981,7 +4978,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -5486,7 +5483,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -5606,7 +5603,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -5615,7 +5612,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -5680,7 +5677,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -6185,7 +6182,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -6305,7 +6302,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -6314,7 +6311,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -6363,7 +6360,7 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
@@ -6379,7 +6376,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -6395,7 +6392,7 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
@@ -6411,7 +6408,7 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
@@ -6654,7 +6651,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="I23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -6666,7 +6663,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="I24" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -6884,7 +6881,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -7004,7 +7001,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -7013,7 +7010,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -7062,7 +7059,7 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
@@ -7078,7 +7075,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -7094,7 +7091,7 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
@@ -7110,7 +7107,7 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
@@ -7353,7 +7350,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="I23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -7365,7 +7362,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="I24" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -7583,7 +7580,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -7703,7 +7700,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -7712,7 +7709,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -7777,7 +7774,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -8282,7 +8279,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -8402,7 +8399,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -8411,7 +8408,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -8476,7 +8473,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -8981,7 +8978,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -9800,7 +9797,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -9809,7 +9806,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -9874,7 +9871,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -10379,7 +10376,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -10499,7 +10496,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -10508,7 +10505,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -10573,7 +10570,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -11078,7 +11075,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -11198,7 +11195,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -11207,7 +11204,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -11272,7 +11269,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -11777,7 +11774,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -11897,7 +11894,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -11906,7 +11903,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -11971,7 +11968,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -12476,7 +12473,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -12596,7 +12593,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -12605,7 +12602,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -12670,7 +12667,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -13175,7 +13172,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -13295,7 +13292,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -13304,7 +13301,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -13369,7 +13366,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -13874,7 +13871,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -13994,7 +13991,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -14003,7 +14000,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -14068,7 +14065,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -14573,7 +14570,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -14693,7 +14690,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -14702,7 +14699,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -14767,7 +14764,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -15272,7 +15269,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -15392,7 +15389,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -15401,7 +15398,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -15466,7 +15463,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -15971,7 +15968,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -16091,7 +16088,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -16100,7 +16097,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -16165,7 +16162,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -16670,7 +16667,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -17489,7 +17486,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -17498,7 +17495,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -17563,7 +17560,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -18068,7 +18065,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -18188,7 +18185,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -18197,7 +18194,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -18262,7 +18259,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -18767,7 +18764,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -18887,7 +18884,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -18896,7 +18893,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -18961,7 +18958,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -19466,7 +19463,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -19586,7 +19583,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -19595,7 +19592,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -19660,7 +19657,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -20165,7 +20162,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -20285,7 +20282,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -20294,7 +20291,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -20359,7 +20356,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -20864,7 +20861,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -20984,7 +20981,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -20993,7 +20990,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -21058,7 +21055,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -21563,7 +21560,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -21683,7 +21680,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -21692,7 +21689,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -21757,7 +21754,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -22262,7 +22259,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -22382,7 +22379,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -22391,7 +22388,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -22456,7 +22453,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -22961,7 +22958,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -23081,7 +23078,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -23090,7 +23087,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -23155,7 +23152,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -23660,7 +23657,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -23780,7 +23777,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -23789,7 +23786,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -23854,7 +23851,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -24359,7 +24356,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -25178,7 +25175,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -25187,7 +25184,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -25252,7 +25249,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -25757,7 +25754,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -25877,7 +25874,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -25886,7 +25883,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -25951,7 +25948,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -26456,7 +26453,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -26576,7 +26573,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -26585,7 +26582,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -26650,7 +26647,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -27155,7 +27152,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -27275,7 +27272,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -27284,7 +27281,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -27349,7 +27346,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -27854,7 +27851,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -28048,7 +28045,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -28064,7 +28061,7 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
@@ -28080,7 +28077,7 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
@@ -28553,7 +28550,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -28747,7 +28744,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -28763,7 +28760,7 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
@@ -28779,7 +28776,7 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
@@ -29252,7 +29249,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -29446,7 +29443,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -29462,7 +29459,7 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
@@ -29478,7 +29475,7 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
@@ -29951,7 +29948,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -30071,7 +30068,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -30080,7 +30077,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -30145,7 +30142,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -30650,7 +30647,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>
@@ -30770,7 +30767,7 @@
         <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -30779,7 +30776,7 @@
         <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -30844,7 +30841,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -31349,7 +31346,7 @@
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G37"/>
       <c r="H37"/>

</xml_diff>